<commit_message>
fix(payroll): include all active field workers regardless of role
</commit_message>
<xml_diff>
--- a/planilha de cadastro de funcionários.xlsx
+++ b/planilha de cadastro de funcionários.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\madri\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\madri\.gemini\antigravity\scratch\daily-log-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A3A3AC8-4447-4278-BDD3-6525C7CED39C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25212442-0D8F-45EF-8509-E78E051402FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{04F5A295-A6F5-4CC1-8434-6A1F8BE7F5F9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="33">
   <si>
     <t>Funcionários, Cargos e Valores</t>
   </si>
@@ -126,13 +126,189 @@
   </si>
   <si>
     <t>formações podem variar dentro da realização de um projeto de acordo com a necessidade da empresa. Por motivos de falta, doença e outras necessidades esta flexibilização precisa existir</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Entendido, anotei o feedback. O Voyager no light mode ficou bom, mas o CSS filter de inversão no dark mode não está funcionando — provavelmente o seletor </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.9"/>
+        <color rgb="FFA31515"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>.dark</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF616161"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> não está alcançando o </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.9"/>
+        <color rgb="FFA31515"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>.leaflet-tile-pane</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF616161"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> porque os estilos </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.9"/>
+        <color rgb="FFA31515"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>jsx global</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF616161"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> do componente não conseguem referenciar a classe </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.9"/>
+        <color rgb="FFA31515"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>.dark</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF616161"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> que está no </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.9"/>
+        <color rgb="FFA31515"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>&lt;html&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF616161"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> ou </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.9"/>
+        <color rgb="FFA31515"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>&lt;body&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF616161"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Quando você quiser que eu corrija, a solução será detectar o tema via JavaScript (observando a classe </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.9"/>
+        <color rgb="FFA31515"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>dark</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF616161"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> no </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.9"/>
+        <color rgb="FFA31515"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>document.documentElement</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF616161"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">) e </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF616161"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>trocar o tile layer programaticamente</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF616161"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> — Voyager no light, CartoDB Dark Matter (ou Positron) no dark — ao invés de depender de CSS filters. Isso é mais confiável que filtros CSS.</t>
+    </r>
+  </si>
+  <si>
+    <t>Aguardo sua instrução para implementar.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -163,6 +339,25 @@
       <color rgb="FF141413"/>
       <name val="Georgia"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF616161"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9.9"/>
+      <color rgb="FFA31515"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF616161"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -243,22 +438,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -277,6 +463,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -612,7 +810,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="908" row="1">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="1">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -634,30 +832,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FFBDC8B-C727-4DD8-8502-EC7043964DF4}">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr defaultColWidth="50.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.85546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="59.140625" style="6" customWidth="1"/>
-    <col min="6" max="6" width="16.7109375" style="6" customWidth="1"/>
-    <col min="7" max="7" width="43.28515625" style="6" customWidth="1"/>
-    <col min="8" max="16384" width="50.5703125" style="6"/>
+    <col min="1" max="1" width="3.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="59.140625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="16.7109375" style="3" customWidth="1"/>
+    <col min="7" max="7" width="43.28515625" style="3" customWidth="1"/>
+    <col min="8" max="8" width="255.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="50.5703125" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:8" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="5"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="11"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -680,300 +879,309 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="A3" s="7">
+    <row r="3" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" s="9" t="s">
+      <c r="D3" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F3" s="10">
+      <c r="F3" s="7">
         <v>1</v>
       </c>
-      <c r="G3" s="11" t="s">
+      <c r="G3" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="A4" s="7">
+    <row r="4" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="A4" s="4">
         <v>2</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4" s="9" t="s">
+      <c r="D4" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F4" s="10">
+      <c r="F4" s="7">
         <v>1</v>
       </c>
-      <c r="G4" s="11" t="s">
+      <c r="G4" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="A5" s="7">
+    <row r="5" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="A5" s="4">
         <v>3</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" s="9" t="s">
+      <c r="D5" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F5" s="10">
+      <c r="F5" s="7">
         <v>1</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="G5" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="A6" s="7">
+    <row r="6" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="A6" s="4">
         <v>4</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E6" s="9" t="s">
+      <c r="D6" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F6" s="10">
+      <c r="F6" s="7">
         <v>2</v>
       </c>
-      <c r="G6" s="11" t="s">
+      <c r="G6" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="A7" s="7">
+    <row r="7" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="A7" s="4">
         <v>5</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E7" s="9" t="s">
+      <c r="D7" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="10">
+      <c r="F7" s="7">
         <v>1</v>
       </c>
-      <c r="G7" s="11" t="s">
+      <c r="G7" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="A8" s="7">
+    <row r="8" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="A8" s="4">
         <v>6</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E8" s="9" t="s">
+      <c r="D8" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F8" s="10">
+      <c r="F8" s="7">
         <v>3</v>
       </c>
-      <c r="G8" s="11" t="s">
+      <c r="G8" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="A9" s="7">
+    <row r="9" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="A9" s="4">
         <v>7</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E9" s="9" t="s">
+      <c r="D9" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F9" s="10">
+      <c r="F9" s="7">
         <v>2</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="G9" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="A10" s="7">
+    <row r="10" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="A10" s="4">
         <v>8</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D10" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E10" s="9" t="s">
+      <c r="D10" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E10" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F10" s="10">
+      <c r="F10" s="7">
         <v>2</v>
       </c>
-      <c r="G10" s="11" t="s">
+      <c r="G10" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="A11" s="7">
-        <v>9</v>
-      </c>
-      <c r="B11" s="8" t="s">
+    <row r="11" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="A11" s="4">
+        <v>9</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E11" s="9" t="s">
+      <c r="D11" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E11" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F11" s="10">
+      <c r="F11" s="7">
         <v>1</v>
       </c>
-      <c r="G11" s="11" t="s">
+      <c r="G11" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="A12" s="7">
+    <row r="12" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="A12" s="4">
         <v>10</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E12" s="9" t="s">
+      <c r="D12" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F12" s="10">
+      <c r="F12" s="7">
         <v>3</v>
       </c>
-      <c r="G12" s="11" t="s">
+      <c r="G12" s="8" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="A13" s="7">
+      <c r="H12" s="12" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="A13" s="4">
         <v>11</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D13" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E13" s="9" t="s">
+      <c r="D13" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E13" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F13" s="10">
+      <c r="F13" s="7">
         <v>2</v>
       </c>
-      <c r="G13" s="11" t="s">
+      <c r="G13" s="8" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="A14" s="7">
+      <c r="H13" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="A14" s="4">
         <v>12</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E14" s="9" t="s">
+      <c r="D14" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F14" s="10">
+      <c r="F14" s="7">
         <v>3</v>
       </c>
-      <c r="G14" s="11" t="s">
+      <c r="G14" s="8" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="7">
+      <c r="H14" s="12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="4">
         <v>13</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E15" s="9" t="s">
+      <c r="D15" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E15" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F15" s="10"/>
-      <c r="G15" s="10"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>